<commit_message>
Restore research prompts and align tutorial
</commit_message>
<xml_diff>
--- a/tutorial/benchmark/ref13-ground-truth.xlsx
+++ b/tutorial/benchmark/ref13-ground-truth.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ref13 benchmark" sheetId="1" r:id="Rff8be2a743b74a74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ref13 benchmark" sheetId="1" r:id="R576a699e852c4d84"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -397,7 +397,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>Ka is the association constant in M^-1. Kd is the reciprocal dissociation constant in µM.</x:v>
+        <x:v>Research schema: Kd (M^-1) is the association constant; K (µM) is the reciprocal dissociation constant.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
@@ -414,16 +414,16 @@
         <x:v>Troponin complex</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
-        <x:v>Measurement</x:v>
+        <x:v>Bound Ca2+ measure</x:v>
       </x:c>
       <x:c r="F5" s="3" t="str">
         <x:v>Mg (mM)</x:v>
       </x:c>
       <x:c r="G5" s="3" t="str">
-        <x:v>Ka (M^-1)</x:v>
+        <x:v>Kd (M^-1)</x:v>
       </x:c>
       <x:c r="H5" s="3" t="str">
-        <x:v>Kd (µM)</x:v>
+        <x:v>K (µM)</x:v>
       </x:c>
     </x:row>
     <x:row r="6">

</xml_diff>